<commit_message>
Update feature tracker with browser test results
</commit_message>
<xml_diff>
--- a/outputs/feature-audit/pearcup-feature-status.xlsx
+++ b/outputs/feature-audit/pearcup-feature-status.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R75715cff1c1349ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" r:id="R715e0a1e6f9d4f10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="3" r:id="Rc8d2b0bc05414627"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="4" r:id="R83f46f538576411a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Map" sheetId="5" r:id="R0bee724ddcb64c3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R614b9c23d5794712"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" r:id="R3fd26402267a4d97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="3" r:id="R27db1ff740834165"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="4" r:id="R3e4c5a4c80f145ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Map" sheetId="5" r:id="R3e855aebee6b45b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -500,8 +500,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestRunsTable" displayName="TestRunsTable" ref="A1:I5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I5"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestRunsTable" displayName="TestRunsTable" ref="A1:I10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I10"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Run ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -750,7 +750,7 @@
     </x:row>
     <x:row r="2" ht="31.5" customHeight="1">
       <x:c r="A2" s="43" t="str">
-        <x:v>Canonical tracker generated from current code after WDK/QVAC integration. Branch: main; commit: 84044b3; generated: 2026-07-02.</x:v>
+        <x:v>Canonical tracker generated from current code after WDK/QVAC integration. Branch: main; commit: d019e18; generated: 2026-07-02.</x:v>
       </x:c>
       <x:c r="B2" s="43"/>
       <x:c r="C2" s="43"/>
@@ -856,7 +856,7 @@
       </x:c>
       <x:c r="B7" s="12" t="n">
         <x:f>COUNTIF('User Stories'!$J$2:$J$200,"Not Run")</x:f>
-        <x:v>54</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
         <x:v>Rows still awaiting manual behavior testing.</x:v>
@@ -883,7 +883,7 @@
       </x:c>
       <x:c r="B8" s="12" t="n">
         <x:f>COUNTIF('User Stories'!$J$2:$J$200,"Passed")+COUNTIF('User Stories'!$J$2:$J$200,"Passed (Smoke)")</x:f>
-        <x:v>16</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
         <x:v>Rows with Passed or Passed (Smoke).</x:v>
@@ -1287,7 +1287,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J2" s="12" t="str">
-        <x:v>Passed (Smoke)</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K2" s="12" t="str"/>
       <x:c r="L2" s="12" t="str">
@@ -1297,7 +1297,7 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N2" s="12" t="str">
-        <x:v>Current live tab passed on 2026-07-02.</x:v>
+        <x:v>Manual browser batches on isolated ports passed clean boot and no console errors.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="45" customHeight="1">
@@ -1371,7 +1371,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J4" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K4" s="12" t="str"/>
       <x:c r="L4" s="12" t="str">
@@ -1380,7 +1380,9 @@
       <x:c r="M4" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N4" s="12" t="str"/>
+      <x:c r="N4" s="12" t="str">
+        <x:v>Reload restored username, Japan team selection, and theme on isolated origin 4178.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="45" customHeight="1">
       <x:c r="A5" s="12" t="str">
@@ -1501,7 +1503,7 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N7" s="12" t="str">
-        <x:v>Head during workbook generation: 84044b3.</x:v>
+        <x:v>Head during workbook generation: d019e18.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="45" customHeight="1">
@@ -1533,7 +1535,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J8" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K8" s="12" t="str"/>
       <x:c r="L8" s="12" t="str">
@@ -1542,7 +1544,9 @@
       <x:c r="M8" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N8" s="12" t="str"/>
+      <x:c r="N8" s="12" t="str">
+        <x:v>Username field accepted codex_tester in browser batch A1.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="45" customHeight="1">
       <x:c r="A9" s="12" t="str">
@@ -1573,7 +1577,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J9" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K9" s="12" t="str"/>
       <x:c r="L9" s="12" t="str">
@@ -1582,7 +1586,9 @@
       <x:c r="M9" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N9" s="12" t="str"/>
+      <x:c r="N9" s="12" t="str">
+        <x:v>Japan team card became selected and persisted through reload.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="45" customHeight="1">
       <x:c r="A10" s="12" t="str">
@@ -1613,7 +1619,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J10" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K10" s="12" t="str"/>
       <x:c r="L10" s="12" t="str">
@@ -1622,7 +1628,9 @@
       <x:c r="M10" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N10" s="12" t="str"/>
+      <x:c r="N10" s="12" t="str">
+        <x:v>Save routed to Home and profile chip showed codex_tester / Japan.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="45" customHeight="1">
       <x:c r="A11" s="12" t="str">
@@ -1653,7 +1661,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J11" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K11" s="12" t="str"/>
       <x:c r="L11" s="12" t="str">
@@ -1662,7 +1670,9 @@
       <x:c r="M11" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N11" s="12" t="str"/>
+      <x:c r="N11" s="12" t="str">
+        <x:v>First-run Kawaii theme selection applied and closed the picker.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="45" customHeight="1">
       <x:c r="A12" s="12" t="str">
@@ -1693,7 +1703,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J12" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K12" s="12" t="str"/>
       <x:c r="L12" s="12" t="str">
@@ -1702,7 +1712,9 @@
       <x:c r="M12" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N12" s="12" t="str"/>
+      <x:c r="N12" s="12" t="str">
+        <x:v>Wallet chip and wallet panel rendered 500 USDT starting balance.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="45" customHeight="1">
       <x:c r="A13" s="12" t="str">
@@ -1733,7 +1745,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J13" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K13" s="12" t="str"/>
       <x:c r="L13" s="12" t="str">
@@ -1742,7 +1754,9 @@
       <x:c r="M13" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N13" s="12" t="str"/>
+      <x:c r="N13" s="12" t="str">
+        <x:v>Fund 50 changed wallet balance from 500 to 550 USDT.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="45" customHeight="1">
       <x:c r="A14" s="12" t="str">
@@ -1773,7 +1787,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J14" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K14" s="12" t="str"/>
       <x:c r="L14" s="12" t="str">
@@ -1782,7 +1796,9 @@
       <x:c r="M14" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N14" s="12" t="str"/>
+      <x:c r="N14" s="12" t="str">
+        <x:v>Collect payouts moved 120 USDT pending payout into balance and marked All collected.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="45" customHeight="1">
       <x:c r="A15" s="12" t="str">
@@ -1853,7 +1869,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J16" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K16" s="12" t="str"/>
       <x:c r="L16" s="12" t="str">
@@ -1862,7 +1878,9 @@
       <x:c r="M16" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N16" s="12" t="str"/>
+      <x:c r="N16" s="12" t="str">
+        <x:v>Live key, match id, and proxy persisted while simulated-feed mode remained disabled.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="45" customHeight="1">
       <x:c r="A17" s="12" t="str">
@@ -1893,7 +1911,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J17" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K17" s="12" t="str"/>
       <x:c r="L17" s="12" t="str">
@@ -1902,7 +1920,9 @@
       <x:c r="M17" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N17" s="12" t="str"/>
+      <x:c r="N17" s="12" t="str">
+        <x:v>Blank API-key test returned Add your API key first.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="45" customHeight="1">
       <x:c r="A18" s="12" t="str">
@@ -1933,7 +1953,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J18" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K18" s="12" t="str"/>
       <x:c r="L18" s="12" t="str">
@@ -1942,7 +1962,9 @@
       <x:c r="M18" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N18" s="12" t="str"/>
+      <x:c r="N18" s="12" t="str">
+        <x:v>Home hero/live area rendered match labels in browser batch A2.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="45" customHeight="1">
       <x:c r="A19" s="12" t="str">
@@ -1973,7 +1995,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J19" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K19" s="12" t="str"/>
       <x:c r="L19" s="12" t="str">
@@ -1982,7 +2004,9 @@
       <x:c r="M19" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N19" s="12" t="str"/>
+      <x:c r="N19" s="12" t="str">
+        <x:v>Overview, Stats, Rooms, Games, and QVAC tabs all activated with content.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="45" customHeight="1">
       <x:c r="A20" s="12" t="str">
@@ -2013,7 +2037,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J20" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K20" s="12" t="str"/>
       <x:c r="L20" s="12" t="str">
@@ -2022,7 +2046,9 @@
       <x:c r="M20" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N20" s="12" t="str"/>
+      <x:c r="N20" s="12" t="str">
+        <x:v>Home rendered four pool cards and four pool CTAs.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="45" customHeight="1">
       <x:c r="A21" s="12" t="str">
@@ -2053,7 +2079,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J21" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K21" s="12" t="str"/>
       <x:c r="L21" s="12" t="str">
@@ -2062,7 +2088,9 @@
       <x:c r="M21" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N21" s="12" t="str"/>
+      <x:c r="N21" s="12" t="str">
+        <x:v>Scoped live fixture CTA opened Watch with Brazil vs Norway.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="45" customHeight="1">
       <x:c r="A22" s="12" t="str">
@@ -2093,7 +2121,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J22" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K22" s="12" t="str"/>
       <x:c r="L22" s="12" t="str">
@@ -2102,7 +2130,9 @@
       <x:c r="M22" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N22" s="12" t="str"/>
+      <x:c r="N22" s="12" t="str">
+        <x:v>Leaderboard panel rendered expected player/prize rows.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="45" customHeight="1">
       <x:c r="A23" s="12" t="str">
@@ -2133,7 +2163,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J23" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K23" s="12" t="str"/>
       <x:c r="L23" s="12" t="str">
@@ -2142,7 +2172,9 @@
       <x:c r="M23" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N23" s="12" t="str"/>
+      <x:c r="N23" s="12" t="str">
+        <x:v>Bracket pool selector and bracket board rendered.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="45" customHeight="1">
       <x:c r="A24" s="12" t="str">
@@ -2173,7 +2205,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J24" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K24" s="12" t="str"/>
       <x:c r="L24" s="12" t="str">
@@ -2182,7 +2214,9 @@
       <x:c r="M24" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N24" s="12" t="str"/>
+      <x:c r="N24" s="12" t="str">
+        <x:v>Focused pool-entry check on port 4179 debited wallet 500 -&gt; 475 and marked $25 pool entered.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="45" customHeight="1">
       <x:c r="A25" s="12" t="str">
@@ -2213,7 +2247,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J25" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K25" s="12" t="str"/>
       <x:c r="L25" s="12" t="str">
@@ -2222,7 +2256,9 @@
       <x:c r="M25" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N25" s="12" t="str"/>
+      <x:c r="N25" s="12" t="str">
+        <x:v>Entrants list included codex_tester after pool entry.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="45" customHeight="1">
       <x:c r="A26" s="12" t="str">
@@ -2253,7 +2289,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J26" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K26" s="12" t="str"/>
       <x:c r="L26" s="12" t="str">
@@ -2262,7 +2298,9 @@
       <x:c r="M26" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N26" s="12" t="str"/>
+      <x:c r="N26" s="12" t="str">
+        <x:v>All 15 bracket picks were selectable with exact forced board clicks and visible as picked.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="45" customHeight="1">
       <x:c r="A27" s="12" t="str">
@@ -2293,7 +2331,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J27" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K27" s="12" t="str"/>
       <x:c r="L27" s="12" t="str">
@@ -2302,7 +2340,9 @@
       <x:c r="M27" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N27" s="12" t="str"/>
+      <x:c r="N27" s="12" t="str">
+        <x:v>Changing r16-1 cleared qf-1, sf-1, and final dependent picks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="45" customHeight="1">
       <x:c r="A28" s="12" t="str">
@@ -2333,7 +2373,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J28" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K28" s="12" t="str"/>
       <x:c r="L28" s="12" t="str">
@@ -2342,7 +2382,9 @@
       <x:c r="M28" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N28" s="12" t="str"/>
+      <x:c r="N28" s="12" t="str">
+        <x:v>Reset cleared all picked team rows.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="45" customHeight="1">
       <x:c r="A29" s="12" t="str">
@@ -2373,7 +2415,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J29" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K29" s="12" t="str"/>
       <x:c r="L29" s="12" t="str">
@@ -2382,7 +2424,9 @@
       <x:c r="M29" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N29" s="12" t="str"/>
+      <x:c r="N29" s="12" t="str">
+        <x:v>Incomplete submit reported 14 picks left and did not complete the bracket.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="45" customHeight="1">
       <x:c r="A30" s="12" t="str">
@@ -2413,7 +2457,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J30" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K30" s="12" t="str"/>
       <x:c r="L30" s="12" t="str">
@@ -2422,7 +2466,9 @@
       <x:c r="M30" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N30" s="12" t="str"/>
+      <x:c r="N30" s="12" t="str">
+        <x:v>Completed bracket submit showed $25 bracket submitted for codex_tester.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="45" customHeight="1">
       <x:c r="A31" s="12" t="str">
@@ -2453,7 +2499,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J31" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K31" s="12" t="str"/>
       <x:c r="L31" s="12" t="str">
@@ -2462,7 +2508,9 @@
       <x:c r="M31" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N31" s="12" t="str"/>
+      <x:c r="N31" s="12" t="str">
+        <x:v>Bracket audit, Tether, runtime, and QVAC panels were present after entry/picks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="45" customHeight="1">
       <x:c r="A32" s="12" t="str">
@@ -2533,7 +2581,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J33" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K33" s="12" t="str"/>
       <x:c r="L33" s="12" t="str">
@@ -2542,7 +2590,9 @@
       <x:c r="M33" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N33" s="12" t="str"/>
+      <x:c r="N33" s="12" t="str">
+        <x:v>Watch TV surface rendered scorebug, pitch, and stats.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="45" customHeight="1">
       <x:c r="A34" s="12" t="str">
@@ -2573,7 +2623,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J34" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K34" s="12" t="str"/>
       <x:c r="L34" s="12" t="str">
@@ -2582,7 +2632,9 @@
       <x:c r="M34" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N34" s="12" t="str"/>
+      <x:c r="N34" s="12" t="str">
+        <x:v>Spanish language tab activated and commentary feed rendered.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="45" customHeight="1">
       <x:c r="A35" s="12" t="str">
@@ -2613,7 +2665,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J35" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="K35" s="12" t="str"/>
       <x:c r="L35" s="12" t="str">
@@ -2622,7 +2674,9 @@
       <x:c r="M35" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N35" s="12" t="str"/>
+      <x:c r="N35" s="12" t="str">
+        <x:v>Simulated feed updated score/stats/commentary. API-only source/live board is intentionally hidden in sim mode and still needs API/relay pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="45" customHeight="1">
       <x:c r="A36" s="12" t="str">
@@ -2653,7 +2707,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J36" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K36" s="12" t="str"/>
       <x:c r="L36" s="12" t="str">
@@ -2662,7 +2716,9 @@
       <x:c r="M36" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N36" s="12" t="str"/>
+      <x:c r="N36" s="12" t="str">
+        <x:v>Chat form appended Testing watch chat to the room feed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="45" customHeight="1">
       <x:c r="A37" s="12" t="str">
@@ -2693,7 +2749,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J37" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K37" s="12" t="str"/>
       <x:c r="L37" s="12" t="str">
@@ -2702,7 +2758,9 @@
       <x:c r="M37" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N37" s="12" t="str"/>
+      <x:c r="N37" s="12" t="str">
+        <x:v>Voice toggle set the live voice state on the control.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="45" customHeight="1">
       <x:c r="A38" s="12" t="str">
@@ -2733,7 +2791,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J38" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K38" s="12" t="str"/>
       <x:c r="L38" s="12" t="str">
@@ -2742,7 +2800,9 @@
       <x:c r="M38" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N38" s="12" t="str"/>
+      <x:c r="N38" s="12" t="str">
+        <x:v>Invite button opened room share bar with pear watch link.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="45" customHeight="1">
       <x:c r="A39" s="12" t="str">
@@ -2813,7 +2873,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J40" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K40" s="12" t="str"/>
       <x:c r="L40" s="12" t="str">
@@ -2822,7 +2882,9 @@
       <x:c r="M40" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N40" s="12" t="str"/>
+      <x:c r="N40" s="12" t="str">
+        <x:v>Reaction button created a reaction pop in the reaction layer.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="45" customHeight="1">
       <x:c r="A41" s="12" t="str">
@@ -2935,7 +2997,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J43" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K43" s="12" t="str"/>
       <x:c r="L43" s="12" t="str">
@@ -2944,7 +3006,9 @@
       <x:c r="M43" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N43" s="12" t="str"/>
+      <x:c r="N43" s="12" t="str">
+        <x:v>Games lobby rendered quick match, four AI challenge buttons, and audit panels.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="45" customHeight="1">
       <x:c r="A44" s="12" t="str">
@@ -2975,7 +3039,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J44" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K44" s="12" t="str"/>
       <x:c r="L44" s="12" t="str">
@@ -2984,7 +3048,9 @@
       <x:c r="M44" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N44" s="12" t="str"/>
+      <x:c r="N44" s="12" t="str">
+        <x:v>Practice vs AI started without wallet debit and exposed the six-zone aim grid.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="45" customHeight="1">
       <x:c r="A45" s="12" t="str">
@@ -3015,7 +3081,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J45" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K45" s="12" t="str"/>
       <x:c r="L45" s="12" t="str">
@@ -3024,7 +3090,9 @@
       <x:c r="M45" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N45" s="12" t="str"/>
+      <x:c r="N45" s="12" t="str">
+        <x:v>Staked Kaito challenge modal accepted, debited 25 USDT, and started a match.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="45" customHeight="1">
       <x:c r="A46" s="12" t="str">
@@ -3055,7 +3123,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J46" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K46" s="12" t="str"/>
       <x:c r="L46" s="12" t="str">
@@ -3064,7 +3132,9 @@
       <x:c r="M46" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N46" s="12" t="str"/>
+      <x:c r="N46" s="12" t="str">
+        <x:v>Friend invite and join-code modals opened with room link/code UI. Two-client convergence remains covered by automated tests.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="45" customHeight="1">
       <x:c r="A47" s="12" t="str">
@@ -3095,7 +3165,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J47" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K47" s="12" t="str"/>
       <x:c r="L47" s="12" t="str">
@@ -3104,7 +3174,9 @@
       <x:c r="M47" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N47" s="12" t="str"/>
+      <x:c r="N47" s="12" t="str">
+        <x:v>Aim-zone kick resolved with banner and HUD update.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="45" customHeight="1">
       <x:c r="A48" s="12" t="str">
@@ -3135,7 +3207,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J48" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K48" s="12" t="str"/>
       <x:c r="L48" s="12" t="str">
@@ -3144,7 +3216,9 @@
       <x:c r="M48" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N48" s="12" t="str"/>
+      <x:c r="N48" s="12" t="str">
+        <x:v>Slower kick sequence progressed HUD through Round 5 of 5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="45" customHeight="1">
       <x:c r="A49" s="12" t="str">
@@ -3175,7 +3249,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J49" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K49" s="12" t="str"/>
       <x:c r="L49" s="12" t="str">
@@ -3184,7 +3258,9 @@
       <x:c r="M49" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N49" s="12" t="str"/>
+      <x:c r="N49" s="12" t="str">
+        <x:v>Shootout reached over state with Back to lobby and Rematch controls.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="45" customHeight="1">
       <x:c r="A50" s="12" t="str">
@@ -3337,7 +3413,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J53" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K53" s="12" t="str"/>
       <x:c r="L53" s="12" t="str">
@@ -3346,7 +3422,9 @@
       <x:c r="M53" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N53" s="12" t="str"/>
+      <x:c r="N53" s="12" t="str">
+        <x:v>Resolver, sync, and replay panels existed after shootout.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="45" customHeight="1">
       <x:c r="A54" s="12" t="str">
@@ -3861,7 +3939,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J66" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K66" s="12" t="str"/>
       <x:c r="L66" s="12" t="str">
@@ -3871,7 +3949,7 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N66" s="12" t="str">
-        <x:v>This is a likely UX-risk area for the next test loop.</x:v>
+        <x:v>Mobile viewport 390x844 activated all primary screens with no page-level horizontal overflow.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="45" customHeight="1">
@@ -4103,7 +4181,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63992fe958024631"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R890cdb8ba5a447c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4833,7 +4911,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34ac2e969a314cbc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ab1a4a792f74b2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4996,6 +5074,151 @@
         <x:v>Server: python3 -m http.server 4175 --bind 127.0.0.1 --directory design/kawaii-app.</x:v>
       </x:c>
     </x:row>
+    <x:row r="6" ht="43.5" customHeight="1">
+      <x:c r="A6" s="12" t="str">
+        <x:v>TR-005</x:v>
+      </x:c>
+      <x:c r="B6" s="29" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="str">
+        <x:v>Profile, Home, wallet, and live settings browser batches</x:v>
+      </x:c>
+      <x:c r="E6" s="12" t="str">
+        <x:v>In-app browser on isolated ports 4178/4179: theme/profile persistence, Home tabs, wallet fund/collect, live setting save/test, fixture CTA</x:v>
+      </x:c>
+      <x:c r="F6" s="12" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G6" s="12" t="str">
+        <x:v>All targeted assertions passed; no browser console errors recorded.</x:v>
+      </x:c>
+      <x:c r="H6" s="12" t="str">
+        <x:v>US-001, US-003, US-007 to US-013, US-015 to US-021, US-023, US-024</x:v>
+      </x:c>
+      <x:c r="I6" s="12" t="str">
+        <x:v>Screen-share permissions were not exercised in this run.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="43.5" customHeight="1">
+      <x:c r="A7" s="12" t="str">
+        <x:v>TR-006</x:v>
+      </x:c>
+      <x:c r="B7" s="29" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="str">
+        <x:v>Bracket board and pool browser batch</x:v>
+      </x:c>
+      <x:c r="E7" s="12" t="str">
+        <x:v>In-app browser on isolated port 4178/4179: pool entry, incomplete submit, reset, 15 picks, downstream clear, completed submit</x:v>
+      </x:c>
+      <x:c r="F7" s="12" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G7" s="12" t="str">
+        <x:v>Pool entry debited 500 -&gt; 475 on focused check; bracket board required exact forced clicks because normal automation click waited on offscreen board rows.</x:v>
+      </x:c>
+      <x:c r="H7" s="12" t="str">
+        <x:v>US-022 to US-030</x:v>
+      </x:c>
+      <x:c r="I7" s="12" t="str">
+        <x:v>Forced clicks were limited to exact bracket team-row selectors after count verification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="43.5" customHeight="1">
+      <x:c r="A8" s="12" t="str">
+        <x:v>TR-007</x:v>
+      </x:c>
+      <x:c r="B8" s="29" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="str">
+        <x:v>Watch party browser batch</x:v>
+      </x:c>
+      <x:c r="E8" s="12" t="str">
+        <x:v>In-app browser on isolated port 4179/4181: Watch screen, language tab, chat, voice, invite, reaction, fixture CTA</x:v>
+      </x:c>
+      <x:c r="F8" s="12" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="G8" s="12" t="str">
+        <x:v>Interactive Watch flows passed. Simulated feed updates stats/commentary; API-only source/live board remains hidden by design and needs API/relay pass.</x:v>
+      </x:c>
+      <x:c r="H8" s="12" t="str">
+        <x:v>US-020, US-032 to US-037, US-039</x:v>
+      </x:c>
+      <x:c r="I8" s="12" t="str">
+        <x:v>Screen share was not clicked because it can trigger browser permission prompts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="43.5" customHeight="1">
+      <x:c r="A9" s="12" t="str">
+        <x:v>TR-008</x:v>
+      </x:c>
+      <x:c r="B9" s="29" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D9" s="12" t="str">
+        <x:v>Penalty Clash browser batch</x:v>
+      </x:c>
+      <x:c r="E9" s="12" t="str">
+        <x:v>In-app browser on isolated ports 4179/4180/4181: practice match, staked challenge, friend invite/join modals, shootout completion</x:v>
+      </x:c>
+      <x:c r="F9" s="12" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G9" s="12" t="str">
+        <x:v>Practice kept wallet unchanged; staked challenge debited 25 USDT; shootout reached over state; friend invite/join modals rendered.</x:v>
+      </x:c>
+      <x:c r="H9" s="12" t="str">
+        <x:v>US-042 to US-048, US-052</x:v>
+      </x:c>
+      <x:c r="I9" s="12" t="str">
+        <x:v>Two-client friend match convergence remains covered by automated worker/P2P tests.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="43.5" customHeight="1">
+      <x:c r="A10" s="12" t="str">
+        <x:v>TR-009</x:v>
+      </x:c>
+      <x:c r="B10" s="29" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="C10" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D10" s="12" t="str">
+        <x:v>Responsive browser sanity</x:v>
+      </x:c>
+      <x:c r="E10" s="12" t="str">
+        <x:v>In-app browser viewport 390x844 across Home, Bracket, Watch, Games, Profile</x:v>
+      </x:c>
+      <x:c r="F10" s="12" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G10" s="12" t="str">
+        <x:v>All primary screens activated with clientWidth 375 and scrollWidth 375; no page-level horizontal overflow.</x:v>
+      </x:c>
+      <x:c r="H10" s="12" t="str">
+        <x:v>US-065</x:v>
+      </x:c>
+      <x:c r="I10" s="12" t="str">
+        <x:v>Topbar wraps tall on mobile but did not overlap content or create horizontal overflow.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F120">
     <x:cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Passed"/>
@@ -5011,7 +5234,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cc8637dede84395"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9150d7e4feb64122"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5251,7 +5474,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ade7177cf9d4815"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R890fa57a1a91407c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update feature audit after full user-story pass
</commit_message>
<xml_diff>
--- a/outputs/feature-audit/pearcup-feature-status.xlsx
+++ b/outputs/feature-audit/pearcup-feature-status.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R614b9c23d5794712"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" r:id="R3fd26402267a4d97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="3" r:id="R27db1ff740834165"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="4" r:id="R3e4c5a4c80f145ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Map" sheetId="5" r:id="R3e855aebee6b45b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rea0d1a33a90c4e2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" r:id="R509abbd43dcf4ce6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="3" r:id="R52f6b8e06a294f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="4" r:id="R11bbed81f6fc4966"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Map" sheetId="5" r:id="R539dba858a224a49"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -500,8 +500,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestRunsTable" displayName="TestRunsTable" ref="A1:I10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I10"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestRunsTable" displayName="TestRunsTable" ref="A1:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Run ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -750,7 +750,7 @@
     </x:row>
     <x:row r="2" ht="31.5" customHeight="1">
       <x:c r="A2" s="43" t="str">
-        <x:v>Canonical tracker generated from current code after WDK/QVAC integration. Branch: main; commit: d019e18; generated: 2026-07-02.</x:v>
+        <x:v>Canonical tracker generated from current code after WDK/QVAC integration. Branch: main; commit: 42abe59; generated: 2026-07-02.</x:v>
       </x:c>
       <x:c r="B2" s="43"/>
       <x:c r="C2" s="43"/>
@@ -814,7 +814,7 @@
         <x:v>Clean</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>git status: main ahead 1 with no dirty files before workbook generation</x:v>
+        <x:v>git status checked before/after commits; no dirty files at handoff expected</x:v>
       </x:c>
       <x:c r="G5" s="12" t="str">
         <x:v>Keep tracker committed after changes.</x:v>
@@ -856,7 +856,7 @@
       </x:c>
       <x:c r="B7" s="12" t="n">
         <x:f>COUNTIF('User Stories'!$J$2:$J$200,"Not Run")</x:f>
-        <x:v>14</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
         <x:v>Rows still awaiting manual behavior testing.</x:v>
@@ -883,7 +883,7 @@
       </x:c>
       <x:c r="B8" s="12" t="n">
         <x:f>COUNTIF('User Stories'!$J$2:$J$200,"Passed")+COUNTIF('User Stories'!$J$2:$J$200,"Passed (Smoke)")</x:f>
-        <x:v>55</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
         <x:v>Rows with Passed or Passed (Smoke).</x:v>
@@ -1413,7 +1413,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J5" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K5" s="12" t="str"/>
       <x:c r="L5" s="12" t="str">
@@ -1422,7 +1422,9 @@
       <x:c r="M5" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N5" s="12" t="str"/>
+      <x:c r="N5" s="12" t="str">
+        <x:v>Demo-mode preflight passed; worker preflight reported demo-locked guard while browser flows continued with demo adapters.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="45" customHeight="1">
       <x:c r="A6" s="12" t="str">
@@ -1453,7 +1455,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J6" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K6" s="12" t="str"/>
       <x:c r="L6" s="12" t="str">
@@ -1462,7 +1464,9 @@
       <x:c r="M6" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N6" s="12" t="str"/>
+      <x:c r="N6" s="12" t="str">
+        <x:v>doctor:live and audit:launch reported QVAC, WDK, compliance, and payout-route blockers without falsely claiming live readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="45" customHeight="1">
       <x:c r="A7" s="12" t="str">
@@ -1503,7 +1507,7 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="N7" s="12" t="str">
-        <x:v>Head during workbook generation: d019e18.</x:v>
+        <x:v>Head during workbook generation: 42abe59.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="45" customHeight="1">
@@ -1829,7 +1833,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J15" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K15" s="12" t="str"/>
       <x:c r="L15" s="12" t="str">
@@ -1838,7 +1842,9 @@
       <x:c r="M15" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N15" s="12" t="str"/>
+      <x:c r="N15" s="12" t="str">
+        <x:v>Negative browser pass withdrew wallet to 0 USDT; paid pool and Kaito stake were blocked with funding-route toasts.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="45" customHeight="1">
       <x:c r="A16" s="12" t="str">
@@ -2541,7 +2547,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J32" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K32" s="12" t="str"/>
       <x:c r="L32" s="12" t="str">
@@ -2550,7 +2556,9 @@
       <x:c r="M32" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N32" s="12" t="str"/>
+      <x:c r="N32" s="12" t="str">
+        <x:v>Entries &amp; payouts panel demo recipient helper saved a 0x route and recipient declarations updated to 2.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="45" customHeight="1">
       <x:c r="A33" s="12" t="str">
@@ -2833,7 +2841,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J39" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="K39" s="12" t="str"/>
       <x:c r="L39" s="12" t="str">
@@ -2842,7 +2850,9 @@
       <x:c r="M39" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N39" s="12" t="str"/>
+      <x:c r="N39" s="12" t="str">
+        <x:v>Manual start/stop requires browser screen-share permission. Not clicked in automation to avoid accepting or triggering capture prompts without user approval.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="45" customHeight="1">
       <x:c r="A40" s="12" t="str">
@@ -2915,7 +2925,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J41" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="K41" s="12" t="str"/>
       <x:c r="L41" s="12" t="str">
@@ -2924,7 +2934,9 @@
       <x:c r="M41" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N41" s="12" t="str"/>
+      <x:c r="N41" s="12" t="str">
+        <x:v>Automated transport/P2P tests pass. In-app browser harness exposed only one active localhost tab, so live BroadcastChannel two-client manual proof was blocked.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="45" customHeight="1">
       <x:c r="A42" s="12" t="str">
@@ -3291,16 +3303,20 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J50" s="12" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K50" s="12" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K50" s="12" t="str">
+        <x:v>DF-001</x:v>
+      </x:c>
       <x:c r="L50" s="12" t="str">
-        <x:v>None</x:v>
+        <x:v>Fixed</x:v>
       </x:c>
       <x:c r="M50" s="12" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="N50" s="12" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="N50" s="12" t="str">
+        <x:v>Header Rematch is now blocked during active staked matches and keeps wallet at 475 USDT; completed-match controls remain visible.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="45" customHeight="1">
       <x:c r="A51" s="12" t="str">
@@ -3331,16 +3347,20 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J51" s="12" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="K51" s="12" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K51" s="12" t="str">
+        <x:v>DF-002</x:v>
+      </x:c>
       <x:c r="L51" s="12" t="str">
-        <x:v>None</x:v>
+        <x:v>Fixed</x:v>
       </x:c>
       <x:c r="M51" s="12" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="N51" s="12" t="str"/>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="N51" s="12" t="str">
+        <x:v>Fresh staked match populated deterministic resolver, QVAC, WDK escrow/payout, receipt, sync, and replay evidence after state-hash and payout-route fix.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="45" customHeight="1">
       <x:c r="A52" s="12" t="str">
@@ -3415,15 +3435,17 @@
       <x:c r="J53" s="12" t="str">
         <x:v>Passed</x:v>
       </x:c>
-      <x:c r="K53" s="12" t="str"/>
+      <x:c r="K53" s="12" t="str">
+        <x:v>DF-002</x:v>
+      </x:c>
       <x:c r="L53" s="12" t="str">
-        <x:v>None</x:v>
+        <x:v>Fixed</x:v>
       </x:c>
       <x:c r="M53" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="N53" s="12" t="str">
-        <x:v>Resolver, sync, and replay panels existed after shootout.</x:v>
+        <x:v>Resolver, sync, replay, QVAC, runtime, and Tether panels populated with event roots and receipt hash after completed staked match.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="45" customHeight="1">
@@ -3455,7 +3477,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J54" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="K54" s="12" t="str"/>
       <x:c r="L54" s="12" t="str">
@@ -3464,7 +3486,9 @@
       <x:c r="M54" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N54" s="12" t="str"/>
+      <x:c r="N54" s="12" t="str">
+        <x:v>Automated P2P lifecycle/forged-event tests pass. Two-client in-app manual challenge was blocked by single-tab harness limitations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="45" customHeight="1">
       <x:c r="A55" s="12" t="str">
@@ -3495,7 +3519,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J55" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="K55" s="12" t="str"/>
       <x:c r="L55" s="12" t="str">
@@ -3504,7 +3528,9 @@
       <x:c r="M55" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N55" s="12" t="str"/>
+      <x:c r="N55" s="12" t="str">
+        <x:v>Friend invite/join modals render and worker/P2P tests pass; live two-tab lobby presence was blocked by in-app single-tab harness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="45" customHeight="1">
       <x:c r="A56" s="12" t="str">
@@ -3739,7 +3765,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J61" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K61" s="12" t="str"/>
       <x:c r="L61" s="12" t="str">
@@ -3748,7 +3774,9 @@
       <x:c r="M61" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N61" s="12" t="str"/>
+      <x:c r="N61" s="12" t="str">
+        <x:v>Watch commentary rendered from live match context and switched to ES without blank/stale feed; worker grounding tests passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="45" customHeight="1">
       <x:c r="A62" s="12" t="str">
@@ -3981,7 +4009,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J67" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K67" s="12" t="str"/>
       <x:c r="L67" s="12" t="str">
@@ -3990,7 +4018,9 @@
       <x:c r="M67" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N67" s="12" t="str"/>
+      <x:c r="N67" s="12" t="str">
+        <x:v>Primary screens had focusable controls, no unnamed enabled buttons, active nav state, and aria-live status toast.</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="45" customHeight="1">
       <x:c r="A68" s="12" t="str">
@@ -4021,7 +4051,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J68" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K68" s="12" t="str"/>
       <x:c r="L68" s="12" t="str">
@@ -4030,7 +4060,9 @@
       <x:c r="M68" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N68" s="12" t="str"/>
+      <x:c r="N68" s="12" t="str">
+        <x:v>Negative API key, incomplete bracket, insufficient funds, and settlement error surfaces all produced actionable recovery/status copy.</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="45" customHeight="1">
       <x:c r="A69" s="12" t="str">
@@ -4101,7 +4133,7 @@
         <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J70" s="12" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K70" s="12" t="str"/>
       <x:c r="L70" s="12" t="str">
@@ -4110,7 +4142,9 @@
       <x:c r="M70" s="12" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="N70" s="12" t="str"/>
+      <x:c r="N70" s="12" t="str">
+        <x:v>preflight:sdk, preflight:worker, preflight:trusted-path, doctor:live, audit:launch, and config:live:print ran; live scripts correctly reported demo/live blockers.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="45" customHeight="1">
       <x:c r="A71" s="12" t="str">
@@ -4129,7 +4163,7 @@
         <x:v>git status; npm run check; design/kawaii-app syntax sweep; in-app browser at 127.0.0.1:4175</x:v>
       </x:c>
       <x:c r="F71" s="12" t="str">
-        <x:v>2026-07-02 checkpoint: main ahead 1, clean; npm run check passed; Kawaii syntax passed; browser smoke passed.</x:v>
+        <x:v>2026-07-02 checkpoints: worktree cleaned between commits; npm run check passed; Kawaii syntax passed; browser smoke passed.</x:v>
       </x:c>
       <x:c r="G71" s="12" t="str">
         <x:v>Run git status, npm run check, Kawaii syntax sweep, and browser top-nav smoke after any fix.</x:v>
@@ -4181,7 +4215,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R890cdb8ba5a447c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03d3bc21e0674799"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4251,36 +4285,92 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
-      <x:c r="A2" s="12" t="str"/>
-      <x:c r="B2" s="12" t="str"/>
-      <x:c r="C2" s="12" t="str"/>
-      <x:c r="D2" s="12" t="str"/>
-      <x:c r="E2" s="12" t="str"/>
-      <x:c r="F2" s="12" t="str"/>
-      <x:c r="G2" s="12" t="str"/>
-      <x:c r="H2" s="12" t="str"/>
-      <x:c r="I2" s="12" t="str"/>
-      <x:c r="J2" s="12" t="str"/>
-      <x:c r="K2" s="12" t="str"/>
-      <x:c r="L2" s="12" t="str"/>
-      <x:c r="M2" s="12" t="str"/>
-      <x:c r="N2" s="12" t="str"/>
+      <x:c r="A2" s="12" t="str">
+        <x:v>DF-001</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="str">
+        <x:v>US-049</x:v>
+      </x:c>
+      <x:c r="C2" s="12" t="str">
+        <x:v>Penalty Clash Gameplay</x:v>
+      </x:c>
+      <x:c r="D2" s="12" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="str">
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="str">
+        <x:v>TR-011</x:v>
+      </x:c>
+      <x:c r="G2" s="12" t="str">
+        <x:v>Header Rematch reset an active staked match without wallet guard.</x:v>
+      </x:c>
+      <x:c r="H2" s="12" t="str">
+        <x:v>Start a staked Kaito match, verify wallet 500 -&gt; 475, click the header Rematch/Spectate control before the match is over.</x:v>
+      </x:c>
+      <x:c r="I2" s="12" t="str">
+        <x:v>Active staked matches cannot be restarted for free; user must finish the match or pay a guarded rematch stake after completion.</x:v>
+      </x:c>
+      <x:c r="J2" s="12" t="str">
+        <x:v>The header control reset the shootout while wallet stayed at 475 USDT, allowing repeated attempts against the same stake.</x:v>
+      </x:c>
+      <x:c r="K2" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="L2" s="12" t="str">
+        <x:v>42abe59</x:v>
+      </x:c>
+      <x:c r="M2" s="12" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="N2" s="12" t="str">
+        <x:v>Retest on port 4185 showed Finish this staked match before starting a rematch and wallet remained 475 USDT.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
-      <x:c r="A3" s="12" t="str"/>
-      <x:c r="B3" s="12" t="str"/>
-      <x:c r="C3" s="12" t="str"/>
-      <x:c r="D3" s="12" t="str"/>
-      <x:c r="E3" s="12" t="str"/>
-      <x:c r="F3" s="12" t="str"/>
-      <x:c r="G3" s="12" t="str"/>
-      <x:c r="H3" s="12" t="str"/>
-      <x:c r="I3" s="12" t="str"/>
-      <x:c r="J3" s="12" t="str"/>
-      <x:c r="K3" s="12" t="str"/>
-      <x:c r="L3" s="12" t="str"/>
-      <x:c r="M3" s="12" t="str"/>
-      <x:c r="N3" s="12" t="str"/>
+      <x:c r="A3" s="12" t="str">
+        <x:v>DF-002</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>US-050, US-052</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="str">
+        <x:v>Game Settlement</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E3" s="12" t="str">
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="F3" s="12" t="str">
+        <x:v>TR-011</x:v>
+      </x:c>
+      <x:c r="G3" s="12" t="str">
+        <x:v>Staked game audit panels stayed on placeholders after the WDK/QVAC worker merge.</x:v>
+      </x:c>
+      <x:c r="H3" s="12" t="str">
+        <x:v>Start and finish a staked Kaito match, then inspect Resolver, Tether WDK, QVAC, P2P sync, and Replay panels.</x:v>
+      </x:c>
+      <x:c r="I3" s="12" t="str">
+        <x:v>Kick and completed-match panels show deterministic resolver, peer state hash evidence, QVAC attestation, WDK escrow/payout, receipt, sync, and replay roots.</x:v>
+      </x:c>
+      <x:c r="J3" s="12" t="str">
+        <x:v>The UI swallowed a settlement exception and left audit panels as Awaiting kick / 0 events placeholders.</x:v>
+      </x:c>
+      <x:c r="K3" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="L3" s="12" t="str">
+        <x:v>42abe59</x:v>
+      </x:c>
+      <x:c r="M3" s="12" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="N3" s="12" t="str">
+        <x:v>Fix submits shooter/keeper state hashes, passes demo payout recipient route, and renders held settlement summaries instead of throwing.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="12" t="str"/>
@@ -4911,7 +5001,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ab1a4a792f74b2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12aeaa9321064979"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5219,6 +5309,151 @@
         <x:v>Topbar wraps tall on mobile but did not overlap content or create horizontal overflow.</x:v>
       </x:c>
     </x:row>
+    <x:row r="11" ht="43.5" customHeight="1">
+      <x:c r="A11" s="12" t="str">
+        <x:v>TR-010</x:v>
+      </x:c>
+      <x:c r="B11" s="29" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="C11" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D11" s="12" t="str">
+        <x:v>Wallet negative and payout recipient browser batch</x:v>
+      </x:c>
+      <x:c r="E11" s="12" t="str">
+        <x:v>In-app browser on isolated port 4182: payout demo recipient save; withdraw to 0; attempt paid pool; attempt staked Kaito challenge</x:v>
+      </x:c>
+      <x:c r="F11" s="12" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G11" s="12" t="str">
+        <x:v>Recipient declarations reached 2; wallet 0 blocked paid pool with Not enough balance; wallet 0 blocked Kaito stake with Need 25 USDT to stake.</x:v>
+      </x:c>
+      <x:c r="H11" s="12" t="str">
+        <x:v>US-014, US-031, US-067</x:v>
+      </x:c>
+      <x:c r="I11" s="12" t="str">
+        <x:v>All checks used visible UI state and toasts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="43.5" customHeight="1">
+      <x:c r="A12" s="12" t="str">
+        <x:v>TR-011</x:v>
+      </x:c>
+      <x:c r="B12" s="29" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="C12" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D12" s="12" t="str">
+        <x:v>Penalty Clash staked settlement regression</x:v>
+      </x:c>
+      <x:c r="E12" s="12" t="str">
+        <x:v>In-app browser on fresh ports 4184/4185: reproduce staked header reset, patch, retest guard, finish staked match, inspect audit panels</x:v>
+      </x:c>
+      <x:c r="F12" s="12" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G12" s="12" t="str">
+        <x:v>Active staked header Rematch blocked with wallet fixed at 475 USDT. Completed Kaito match showed deterministic resolver, QVAC attestation, WDK escrow/payout, receipt hash, matched sync roots, and replay log.</x:v>
+      </x:c>
+      <x:c r="H12" s="12" t="str">
+        <x:v>US-049, US-050, US-052</x:v>
+      </x:c>
+      <x:c r="I12" s="12" t="str">
+        <x:v>Fix added guarded restart, peer state-hash submissions, demo payout recipient route, and held-summary panel protection.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="43.5" customHeight="1">
+      <x:c r="A13" s="12" t="str">
+        <x:v>TR-012</x:v>
+      </x:c>
+      <x:c r="B13" s="29" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="C13" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D13" s="12" t="str">
+        <x:v>Release preflight scripts</x:v>
+      </x:c>
+      <x:c r="E13" s="12" t="str">
+        <x:v>npm run preflight:sdk; npm run preflight:worker; npm run preflight:trusted-path; npm run doctor:live; npm run audit:launch; npm run config:live:print</x:v>
+      </x:c>
+      <x:c r="F13" s="12" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G13" s="12" t="str">
+        <x:v>SDK and trusted-path preflights passed. Worker stayed demo-locked. Live doctor and launch audit reported QVAC/WDK/compliance/payout blockers without claiming live readiness.</x:v>
+      </x:c>
+      <x:c r="H13" s="12" t="str">
+        <x:v>US-041, US-063, US-069, US-070</x:v>
+      </x:c>
+      <x:c r="I13" s="12" t="str">
+        <x:v>audit:launch intentionally reports blocked live launch in demo config.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="43.5" customHeight="1">
+      <x:c r="A14" s="12" t="str">
+        <x:v>TR-013</x:v>
+      </x:c>
+      <x:c r="B14" s="29" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="str">
+        <x:v>Accessibility and QVAC commentary browser pass</x:v>
+      </x:c>
+      <x:c r="E14" s="12" t="str">
+        <x:v>In-app browser on isolated app tab: scan primary screens for unlabeled enabled buttons/focusable controls; switch Watch commentary to ES</x:v>
+      </x:c>
+      <x:c r="F14" s="12" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="G14" s="12" t="str">
+        <x:v>Profile/Home/Bracket/Watch/Games had focusable controls, no unnamed enabled buttons, active nav, and aria-live toast. ES commentary rendered from live match feed.</x:v>
+      </x:c>
+      <x:c r="H14" s="12" t="str">
+        <x:v>US-060, US-066</x:v>
+      </x:c>
+      <x:c r="I14" s="12" t="str">
+        <x:v>This was a fast accessibility sanity pass, not a full assistive-technology audit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="43.5" customHeight="1">
+      <x:c r="A15" s="12" t="str">
+        <x:v>TR-014</x:v>
+      </x:c>
+      <x:c r="B15" s="29" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="str">
+        <x:v>Peer and screen-share manual blockers</x:v>
+      </x:c>
+      <x:c r="E15" s="12" t="str">
+        <x:v>Attempted same-origin two-tab in-app browser peer lobby on port 4186; reviewed screen-share permission path</x:v>
+      </x:c>
+      <x:c r="F15" s="12" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="G15" s="12" t="str">
+        <x:v>In-app browser exposed only one active localhost tab for the 4186 origin, so BroadcastChannel two-client manual convergence could not be proven there. Screen share requires user-controlled browser capture permission.</x:v>
+      </x:c>
+      <x:c r="H15" s="12" t="str">
+        <x:v>US-038, US-040, US-053, US-054</x:v>
+      </x:c>
+      <x:c r="I15" s="12" t="str">
+        <x:v>Automated worker, transport, peer lifecycle, and forged-event tests passed under npm run check.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F120">
     <x:cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Passed"/>
@@ -5234,7 +5469,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9150d7e4feb64122"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b940759e4f54ddf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5474,7 +5709,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R890fa57a1a91407c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a351b3953554208"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>